<commit_message>
chore(repo): el trabajo local de agosto llega a GitHub
Cola de producción, orden del catálogo, numeración de pedidos, corte del Excel Lover y el backlog al día (Singapur, Nueva York, contraseñas). Fuera quedan los ficheros que git marca cambiados y el diff deja vacíos.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/plantillas/plantilla-materiales.xlsx
+++ b/docs/plantillas/plantilla-materiales.xlsx
@@ -345,14 +345,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="U1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">Opcional. 1 deja el material activo, 0 lo oculta de listados (Inactive). Vacio = activo. OJO: escribir "Inactive" cuenta como 1.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="198">
-  <si>
-    <t>Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="203">
+  <si>
+    <t>Material name</t>
   </si>
   <si>
     <t>Material Type</t>
@@ -361,7 +377,7 @@
     <t>Supplier</t>
   </si>
   <si>
-    <t>Purchase Cost</t>
+    <t>Purchase Cost (No VAT)</t>
   </si>
   <si>
     <t>Purchase UoM</t>
@@ -382,7 +398,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Traceability</t>
+    <t>Traceable</t>
   </si>
   <si>
     <t>Colors</t>
@@ -391,19 +407,19 @@
     <t>Internal SKU</t>
   </si>
   <si>
-    <t>Importer Item ID</t>
+    <t>Importer item ID</t>
   </si>
   <si>
     <t>Supplier Lead Time (Days)</t>
   </si>
   <si>
-    <t>Minimum Order Quantity (MOQ)</t>
-  </si>
-  <si>
-    <t>Reorder Point (ROP)</t>
-  </si>
-  <si>
-    <t>Safety Stock Qty</t>
+    <t>MOQ (UoP)</t>
+  </si>
+  <si>
+    <t>Reorder Point (ROP) (UoS)</t>
+  </si>
+  <si>
+    <t>Safety Stock Qty (UoS)</t>
   </si>
   <si>
     <t>Scrap / Loss Margin (%)</t>
@@ -412,6 +428,9 @@
     <t>Volume per Purchase UoM (CBM)</t>
   </si>
   <si>
+    <t>Active</t>
+  </si>
+  <si>
     <t>Leather Cowhide Black 1.2mm</t>
   </si>
   <si>
@@ -553,7 +572,7 @@
     <t>Plantilla de importacion de materiales - ANV Fight Gear</t>
   </si>
   <si>
-    <t>Generada el 2026-08-15 13:07 leyendo el importador tec_inventory_csv_importer.</t>
+    <t>Generada el 2026-08-20 02:08 leyendo el importador tec_inventory_csv_importer.</t>
   </si>
   <si>
     <t>Los nombres de columna de la hoja Materiales son los que el importador espera. No se cambian.</t>
@@ -574,7 +593,7 @@
     <t>4. Subir en /feed/4/import, la ficha "Inventory Excel-CSV file".</t>
   </si>
   <si>
-    <t>Tres cosas que hacen fallar la importacion en silencio</t>
+    <t>Cosas que hacen fallar la importacion en silencio</t>
   </si>
   <si>
     <t>- Coma decimal. El importador quiere punto: 1850.50, no 1850,50. Con coma el numero entra vacio.</t>
@@ -583,7 +602,10 @@
     <t>- Espacios sobrantes en las columnas de lista. "Blue " con un espacio detras no encuentra "Blue".</t>
   </si>
   <si>
-    <t>- La columna Traceability: solo 1, 0 o vacio. Escribir "No" cuenta como 1.</t>
+    <t>- La columna Traceable: solo 1, 0 o vacio. Escribir "No" cuenta como 1.</t>
+  </si>
+  <si>
+    <t>- La columna Active: solo 1, 0 o vacio. Vacio deja el material activo. Escribir "Inactive" cuenta como 1.</t>
   </si>
   <si>
     <t>Que pasa si un valor de lista no existe</t>
@@ -760,6 +782,12 @@
     <t>Metros cubicos que ocupa una unidad de compra. Para calcular el flete.</t>
   </si>
   <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>1 deja el material activo, 0 lo oculta de listados (Inactive). Vacio = activo. OJO: escribir "Inactive" cuenta como 1.</t>
+  </si>
+  <si>
     <t>Unidades que existen hoy (13)</t>
   </si>
   <si>
@@ -943,7 +971,10 @@
     <t>Yellow</t>
   </si>
   <si>
-    <t>Proveedores que existen hoy (1)</t>
+    <t>Proveedores que existen hoy (2)</t>
+  </si>
+  <si>
+    <t>POLYTEC ASIA COMPANY LIMITED co.,ltd.</t>
   </si>
 </sst>
 </file>
@@ -1373,32 +1404,33 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="true" style="0"/>
+    <col min="1" max="1" width="17" customWidth="true" style="0"/>
     <col min="2" max="2" width="17" customWidth="true" style="0"/>
     <col min="3" max="3" width="14" customWidth="true" style="0"/>
-    <col min="4" max="4" width="17" customWidth="true" style="0"/>
+    <col min="4" max="4" width="26" customWidth="true" style="0"/>
     <col min="5" max="5" width="16" customWidth="true" style="0"/>
     <col min="6" max="6" width="17" customWidth="true" style="0"/>
     <col min="7" max="7" width="19" customWidth="true" style="0"/>
     <col min="8" max="8" width="32" customWidth="true" style="0"/>
     <col min="9" max="9" width="34" customWidth="true" style="0"/>
     <col min="10" max="10" width="15" customWidth="true" style="0"/>
-    <col min="11" max="11" width="16" customWidth="true" style="0"/>
+    <col min="11" max="11" width="14" customWidth="true" style="0"/>
     <col min="12" max="12" width="14" customWidth="true" style="0"/>
     <col min="13" max="13" width="16" customWidth="true" style="0"/>
     <col min="14" max="14" width="20" customWidth="true" style="0"/>
     <col min="15" max="15" width="29" customWidth="true" style="0"/>
-    <col min="16" max="16" width="32" customWidth="true" style="0"/>
-    <col min="17" max="17" width="23" customWidth="true" style="0"/>
-    <col min="18" max="18" width="20" customWidth="true" style="0"/>
+    <col min="16" max="16" width="14" customWidth="true" style="0"/>
+    <col min="17" max="17" width="29" customWidth="true" style="0"/>
+    <col min="18" max="18" width="26" customWidth="true" style="0"/>
     <col min="19" max="19" width="27" customWidth="true" style="0"/>
     <col min="20" max="20" width="33" customWidth="true" style="0"/>
+    <col min="21" max="21" width="14" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" customHeight="1" ht="34">
+    <row r="1" spans="1:21" customHeight="1" ht="34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1459,191 +1491,203 @@
       <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:20">
+      <c r="U1" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21">
       <c r="A2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="D3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" s="5" t="s">
+    </row>
+    <row r="4" spans="1:21">
+      <c r="A4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20">
-      <c r="A3" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" s="5" t="s">
+      <c r="M4" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="R4" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="K3" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20">
-      <c r="A4" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>44</v>
-      </c>
       <c r="S4" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1659,7 +1703,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="true" style="0"/>
@@ -1670,7 +1714,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D1" s="8"/>
     </row>
@@ -1679,13 +1723,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D3" s="8"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D4" s="8"/>
     </row>
@@ -1694,31 +1738,31 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6" s="8"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D7" s="8"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D8" s="8"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D9" s="8"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D10" s="8"/>
     </row>
@@ -1727,155 +1771,147 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D12" s="8"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D13" s="8"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D14" s="8"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D15" s="8"/>
     </row>
     <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>79</v>
+      </c>
       <c r="D16" s="8"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>79</v>
+      <c r="A18" s="7" t="s">
+        <v>80</v>
       </c>
       <c r="D18" s="8"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D19" s="8"/>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D20" s="8"/>
     </row>
     <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>83</v>
+      </c>
       <c r="D21" s="8"/>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="7" t="s">
-        <v>82</v>
-      </c>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>83</v>
+      <c r="A23" s="7" t="s">
+        <v>84</v>
       </c>
       <c r="D23" s="8"/>
     </row>
     <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>85</v>
+      </c>
       <c r="D24" s="8"/>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="7" t="s">
-        <v>84</v>
-      </c>
       <c r="D25" s="8"/>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" t="s">
-        <v>85</v>
+      <c r="A26" s="7" t="s">
+        <v>86</v>
       </c>
       <c r="D26" s="8"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D27" s="8"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D28" s="8"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D29" s="8"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D30" s="8"/>
     </row>
     <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>91</v>
+      </c>
       <c r="D31" s="8"/>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="7" t="s">
-        <v>90</v>
-      </c>
       <c r="D32" s="8"/>
     </row>
     <row r="33" spans="1:4">
+      <c r="A33" s="7" t="s">
+        <v>92</v>
+      </c>
       <c r="D33" s="8"/>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="8"/>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="B35" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C36" t="s">
         <v>98</v>
@@ -1886,10 +1922,10 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C37" t="s">
         <v>100</v>
@@ -1900,10 +1936,10 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C38" t="s">
         <v>102</v>
@@ -1914,10 +1950,10 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C39" t="s">
         <v>104</v>
@@ -1928,10 +1964,10 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C40" t="s">
         <v>106</v>
@@ -1942,10 +1978,10 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C41" t="s">
         <v>108</v>
@@ -1956,10 +1992,10 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C42" t="s">
         <v>110</v>
@@ -1970,10 +2006,10 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C43" t="s">
         <v>112</v>
@@ -1983,8 +2019,11 @@
       </c>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" t="s">
-        <v>9</v>
+      <c r="A44" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>97</v>
       </c>
       <c r="C44" t="s">
         <v>114</v>
@@ -1995,7 +2034,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C45" t="s">
         <v>116</v>
@@ -2006,7 +2045,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C46" t="s">
         <v>118</v>
@@ -2017,7 +2056,7 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C47" t="s">
         <v>120</v>
@@ -2028,7 +2067,7 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C48" t="s">
         <v>122</v>
@@ -2039,7 +2078,7 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C49" t="s">
         <v>124</v>
@@ -2050,7 +2089,7 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C50" t="s">
         <v>126</v>
@@ -2061,7 +2100,7 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C51" t="s">
         <v>128</v>
@@ -2072,7 +2111,7 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C52" t="s">
         <v>130</v>
@@ -2083,7 +2122,7 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C53" t="s">
         <v>132</v>
@@ -2094,7 +2133,7 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C54" t="s">
         <v>134</v>
@@ -2104,7 +2143,29 @@
       </c>
     </row>
     <row r="55" spans="1:4">
-      <c r="D55" s="8"/>
+      <c r="A55" t="s">
+        <v>19</v>
+      </c>
+      <c r="C55" t="s">
+        <v>136</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" t="s">
+        <v>20</v>
+      </c>
+      <c r="C56" t="s">
+        <v>138</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="D57" s="8"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
@@ -2126,72 +2187,72 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="9" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="10" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2214,117 +2275,117 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="9" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="10" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="10" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="10" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="10" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="10" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="10" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="10" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="10" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="10" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="10" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="10" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="10" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="10" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="10" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="10" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="10" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2347,167 +2408,167 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="9" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="10" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="10" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="10" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="10" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="10" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="10" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="10" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="10" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="10" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="10" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="10" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="10" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="10" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="10" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="10" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="10" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="10" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="10" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="10" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" s="10" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="10" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="10" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="10" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="10" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="10" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="10" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" s="10" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="10" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" s="10" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2522,7 +2583,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="true" style="0"/>
@@ -2530,12 +2591,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="9" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="10" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>